<commit_message>
Final commit of selenium python
</commit_message>
<xml_diff>
--- a/saucedemo_python/data/login_data.xlsx
+++ b/saucedemo_python/data/login_data.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="valid_data" sheetId="1" r:id="rId1"/>
-    <sheet name="invalid_data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>Username</t>
   </si>
@@ -43,15 +42,6 @@
   </si>
   <si>
     <t>locked_out_user</t>
-  </si>
-  <si>
-    <t>wrong_password</t>
-  </si>
-  <si>
-    <t>admin</t>
-  </si>
-  <si>
-    <t>password123</t>
   </si>
 </sst>
 </file>
@@ -1239,44 +1229,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="1"/>
-  <cols>
-    <col min="1" max="1" width="21.1428571428571" customWidth="1"/>
-    <col min="2" max="2" width="21.5714285714286" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
 </file>
</xml_diff>